<commit_message>
Remplace l'ancien slogan par « food truck local, végétal et gourmand »
Mentionne les légumes de saison du potager et les produits bio autant que possible (page événements, plaquette, modèles d'e-mails, notes projet).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZLSKwfEZhmFaHDXKS8XKA
</commit_message>
<xml_diff>
--- a/prospection/Yummy_Prospection_Evenements.xlsx
+++ b/prospection/Yummy_Prospection_Evenements.xlsx
@@ -2786,7 +2786,7 @@
 Toutes nos formules : https://yummy-streetfood.be/evenements-prives?src=lieux
 Belle journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2811,7 +2811,7 @@
 Notre offre mariage : https://yummy-streetfood.be/evenements-prives?src=planners
 Au plaisir,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2840,7 +2840,7 @@
 Et pour un devis en deux minutes : https://yummy-streetfood.be/evenements-prives?src=entreprises
 Bonne journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2865,7 +2865,7 @@
 Nos formules : https://yummy-streetfood.be/evenements-prives?src=communes
 Merci d'avance et belle journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2890,7 +2890,7 @@
 Lien direct pour vos clients : https://yummy-streetfood.be/evenements-prives?src=gites
 Belle journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2915,7 +2915,7 @@
 Nos formules : https://yummy-streetfood.be/evenements-prives?src=reseaux
 Au plaisir d'échanger,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2937,7 +2937,7 @@
 Je me permets de revenir vers vous au sujet de mon message de la semaine dernière. Notre proposition de passer vous faire goûter nos starters tient toujours, cela prend dix minutes.
 Bonne journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2959,7 +2959,7 @@
 Dernier petit message de ma part, promis ! Si ce n'est pas le bon moment, aucun souci : je garde vos coordonnées et vous recontacterai au printemps. Et si un événement se présente d'ici là, vous savez où nous trouver.
 Belle continuation,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -2984,7 +2984,7 @@
 2. Penser à nous si quelqu'un autour de vous prépare un mariage, un anniversaire ou une fête d'entreprise. Pour chaque événement réservé grâce à vous, {cadeau parrainage}.
 À bientôt sur les marchés,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>
@@ -3009,7 +3009,7 @@
 Si vous voulez goûter avant de décider, venez nous voir au marché (Virton le vendredi, Arlon le jeudi, de 8 h à 13 h).
 Belle journée,
 Christelle &amp; Thomas
-Yummy Street Food — la street-food cultivée par la maraîchère
+Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Reformule les starters (formule 3 ou 5), remplace « snack », objets « sur mesure », signature Christelle Muller
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZLSKwfEZhmFaHDXKS8XKA
</commit_message>
<xml_diff>
--- a/prospection/Yummy_Prospection_Evenements.xlsx
+++ b/prospection/Yummy_Prospection_Evenements.xlsx
@@ -2773,19 +2773,19 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Prestataire street food végétale pour vos mariages et réceptions ?</t>
+          <t>Prestation food truck sur mesure pour vos mariages et réceptions</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Bonjour,
 Nous sommes Yummy Street Food, le food truck vert de Virton : une street-food végétale préparée avec les légumes que nous cultivons nous-mêmes.
-Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail dans votre parc, nos 5 starters à 3 € pièce plaisent beaucoup, et en fin de soirée, un snack street food sorti de la remorque fait toujours son effet.
+Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail, nous proposons une formule de 3 ou 5 starters végétaux, puis nos plats street food (burgers, pitas, wraps, bowls), et même un service en fin de soirée.
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Le plus simple est encore de goûter : nous pouvons passer vous déposer un plateau de starters, à vous de nous dire quand.
 Toutes nos formules : https://yummy-streetfood.be/evenements-prives?src=lieux
 Belle journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2799,18 +2799,18 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Une idée food truck végétal pour vos mariés</t>
+          <t>Une prestation food truck sur mesure pour vos mariés</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Bonjour {prénom},
 J'ai découvert votre travail et votre approche des mariages, et je pense que nous pourrions faire de beaux mariages ensemble.
-Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : bowls fleuris, pitas, starters à l'apéro, avec les légumes de notre potager en Gaume. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
+Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : bowls fleuris, pitas, starters en ouverture, avec les légumes de notre potager en Gaume. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
 Seriez-vous partant(e) pour un café et une dégustation ? Et bien sûr, nous recommandons volontiers vos services à nos clients en retour.
 Notre offre mariage : https://yummy-streetfood.be/evenements-prives?src=planners
 Au plaisir,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fête du personnel ou family day : un food truck local pour vos équipes</t>
+          <t>Prestation food truck sur mesure pour vos événements d'entreprise</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2834,12 +2834,12 @@
 Yummy Street Food est un food truck basé à Virton. Nous cuisinons une street-food végétale et gourmande avec les légumes de notre propre potager. Concrètement, la remorque s'installe sur votre site et sert vos équipes rapidement, sans qu'il y ait rien à organiser de votre côté.
 Nous proposons par exemple :
 - un lunch d'équipe ou une pause midi sur le parking ;
-- un apéro avec nos 5 starters à 3 € pièce ;
+- un apéro avec une formule de 3 ou 5 starters végétaux ;
 - un repas complet pour une fête du personnel ou un family day.
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Et pour un devis en deux minutes : https://yummy-streetfood.be/evenements-prives?src=entreprises
 Bonne journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2864,7 +2864,7 @@
 Nous serions aussi ravis de participer aux événements organisés par la commune.
 Nos formules : https://yummy-streetfood.be/evenements-prives?src=communes
 Merci d'avance et belle journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2878,18 +2878,18 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Une soirée food truck pour vos groupes ?</t>
+          <t>Une soirée food truck sur mesure pour vos groupes</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Bonjour,
 Vos gîtes accueillent des groupes pour des anniversaires, des week-ends entre amis ou des réunions de famille. Pour eux, la question du repas du samedi soir revient souvent.
-Nous sommes Yummy Street Food, un food truck végétal et local basé à Virton, à quelques minutes de chez vous. Nous pouvons venir cuisiner sur place pour vos hôtes (starters à l'apéro, pitas, burgers, bowls).
+Nous sommes Yummy Street Food, un food truck végétal et local basé à Virton, à quelques minutes de chez vous. Nous pouvons venir cuisiner sur place pour vos hôtes (starters à l'apéro, puis burgers, pitas ou bowls).
 Seriez-vous d'accord de mentionner cette option à vos clients ? Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Lien direct pour vos clients : https://yummy-streetfood.be/evenements-prives?src=gites
 Belle journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2914,7 +2914,7 @@
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Nos formules : https://yummy-streetfood.be/evenements-prives?src=reseaux
 Au plaisir d'échanger,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2936,7 +2936,7 @@
           <t>Bonjour,
 Je me permets de revenir vers vous au sujet de mon message de la semaine dernière. Notre proposition de passer vous faire goûter nos starters tient toujours, cela prend dix minutes.
 Bonne journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2958,7 +2958,7 @@
           <t>Bonjour,
 Dernier petit message de ma part, promis ! Si ce n'est pas le bon moment, aucun souci : je garde vos coordonnées et vous recontacterai au printemps. Et si un événement se présente d'ici là, vous savez où nous trouver.
 Belle continuation,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -2983,7 +2983,7 @@
 1. Laisser un avis Google (deux minutes) : {lien avis Google}
 2. Penser à nous si quelqu'un autour de vous prépare un mariage, un anniversaire ou une fête d'entreprise. Pour chaque événement réservé grâce à vous, {cadeau parrainage}.
 À bientôt sur les marchés,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -3008,7 +3008,7 @@
 Ce prix comprend la venue de la remorque, la préparation sur place et le service. Pour bloquer la date, il suffit de nous confirmer par retour de mail.
 Si vous voulez goûter avant de décider, venez nous voir au marché (Virton le vendredi, Arlon le jeudi, de 8 h à 13 h).
 Belle journée,
-Christelle &amp; Thomas
+Christelle Muller
 Yummy Street Food — food truck local, végétal et gourmand
 +32 474 60 64 51 · yummy-streetfood.be</t>
         </is>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>« Bonjour, Christelle [ou Thomas] de Yummy Street Food, le food truck végétal de Virton. Je vous ai envoyé un petit mail la semaine dernière. Je vous appelle juste pour savoir à qui je dois m'adresser pour les [fêtes du personnel / mariages chez vous]. »
+          <t>« Bonjour, Christelle Muller de Yummy Street Food, le food truck végétal de Virton. Je vous ai envoyé un petit mail la semaine dernière. Je vous appelle juste pour savoir à qui je dois m'adresser pour les [fêtes du personnel / mariages chez vous]. »
 → Si intéressé : « Le plus simple, c'est que je passe vous faire goûter nos starters. Plutôt mardi ou jeudi ? »
 → Si pas le moment : « Aucun souci. Je peux vous rappeler quand ? En janvier pour les événements de printemps ? » (noter la date dans « Prochaine relance »)</t>
         </is>

</xml_diff>

<commit_message>
Formules événements : La Complète, La Gourmande, L'Essentielle (dessert en option), photo burger
- Section « Une prestation sur mesure » en liste claire sur la page et la plaquette
- Plat street food : burger ou pita ; dessert ajouté au calculateur de devis

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZLSKwfEZhmFaHDXKS8XKA
</commit_message>
<xml_diff>
--- a/prospection/Yummy_Prospection_Evenements.xlsx
+++ b/prospection/Yummy_Prospection_Evenements.xlsx
@@ -664,7 +664,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>• Onglet « Devis » : vos prix (plat, boissons, déplacement, minimum de prestation). Seul le prix des starters (3 €) est connu à ce jour.</t>
+          <t>• Onglet « Devis » : vos prix (plat, dessert, boissons, déplacement, minimum de prestation). Seul le prix des starters (3 €) est connu à ce jour.</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
         <is>
           <t>Bonjour,
 Nous sommes Yummy Street Food, le food truck vert de Virton : une street-food végétale préparée avec les légumes que nous cultivons nous-mêmes.
-Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail, nous proposons une formule de 3 ou 5 starters végétaux, puis nos plats street food (burgers, pitas, wraps, bowls), et même un service en fin de soirée.
+Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail, nous proposons une formule de 3 ou 5 starters végétaux, puis un plat street food (burger ou pita) et un dessert si vous le souhaitez. Nous pouvons aussi assurer un service en fin de soirée.
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Le plus simple est encore de goûter : nous pouvons passer vous déposer un plateau de starters, à vous de nous dire quand.
 Toutes nos formules : https://yummy-streetfood.be/evenements-prives?src=lieux
@@ -2806,7 +2806,7 @@
         <is>
           <t>Bonjour {prénom},
 J'ai découvert votre travail et votre approche des mariages, et je pense que nous pourrions faire de beaux mariages ensemble.
-Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : bowls fleuris, pitas, starters en ouverture, avec les légumes de notre potager en Gaume. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
+Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : starters en ouverture, puis burgers et pitas, avec les légumes de notre potager en Gaume. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
 Seriez-vous partant(e) pour un café et une dégustation ? Et bien sûr, nous recommandons volontiers vos services à nos clients en retour.
 Notre offre mariage : https://yummy-streetfood.be/evenements-prives?src=planners
 Au plaisir,
@@ -2885,7 +2885,7 @@
         <is>
           <t>Bonjour,
 Vos gîtes accueillent des groupes pour des anniversaires, des week-ends entre amis ou des réunions de famille. Pour eux, la question du repas du samedi soir revient souvent.
-Nous sommes Yummy Street Food, un food truck végétal et local basé à Virton, à quelques minutes de chez vous. Nous pouvons venir cuisiner sur place pour vos hôtes (starters à l'apéro, puis burgers, pitas ou bowls).
+Nous sommes Yummy Street Food, un food truck végétal et local basé à Virton, à quelques minutes de chez vous. Nous pouvons venir cuisiner sur place pour vos hôtes (starters à l'apéro, puis burger ou pita, et un dessert).
 Seriez-vous d'accord de mentionner cette option à vos clients ? Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Lien direct pour vos clients : https://yummy-streetfood.be/evenements-prives?src=gites
 Belle journée,
@@ -3507,7 +3507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3541,15 +3541,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Starters par invité</t>
+          <t>Starters par invité (0, 3 ou 5)</t>
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Apéro / vin d'honneur</t>
+          <t>La Complète = 5 · La Gourmande = 3 · L'Essentielle = 0</t>
         </is>
       </c>
     </row>
@@ -3562,22 +3562,22 @@
       <c r="B4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Connu : 3 € pièce</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Plat principal ? (1 = oui, 0 = non)</t>
+          <t>Plat street food ? (1 = oui, 0 = non)</t>
         </is>
       </c>
       <c r="B5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Burger ou pita</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3595,109 +3595,149 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Boissons par invité (€)</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n"/>
+          <t>Dessert ? (1 = oui, 0 = non)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>À FIXER (0 si pas de boissons)</t>
+          <t>En option sur La Complète et La Gourmande, inclus dans L'Essentielle</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Forfait déplacement (€)</t>
+          <t>Prix du dessert par invité (€)</t>
         </is>
       </c>
       <c r="B8" s="11" t="n"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>À FIXER (ex. selon la distance depuis Virton)</t>
+          <t>À FIXER par vous</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Minimum de prestation (€)</t>
+          <t>Boissons par invité (€)</t>
         </is>
       </c>
       <c r="B9" s="11" t="n"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>À FIXER (repère du marché : 250 à 800 €)</t>
+          <t>À FIXER (0 si pas de boissons)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Forfait déplacement (€)</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>À FIXER (ex. selon la distance depuis Virton)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Minimum de prestation (€)</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>À FIXER (repère du marché : 250 à 800 €)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Sous-total starters</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B13">
         <f>B2*B3*B4</f>
         <v/>
       </c>
-      <c r="C11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Sous-total plats</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B14">
         <f>B2*B5*B6</f>
         <v/>
       </c>
-      <c r="C12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sous-total desserts</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B2*B7*B8</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Sous-total boissons</t>
         </is>
       </c>
-      <c r="B13">
-        <f>B2*B7</f>
+      <c r="B16">
+        <f>B2*B9</f>
         <v/>
       </c>
-      <c r="C13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>TOTAL PROPOSÉ (€)</t>
         </is>
       </c>
-      <c r="B14" s="13">
-        <f>MAX(B9,B11+B12+B13+B8)</f>
+      <c r="B17" s="13">
+        <f>MAX(B11,B13+B14+B15+B16+B10)</f>
         <v/>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Le minimum de prestation s'applique si le total est inférieur</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Prix par invité (€)</t>
         </is>
       </c>
-      <c r="B15" s="13">
-        <f>IF(B2&gt;0,B14/B2,0)</f>
+      <c r="B18" s="13">
+        <f>IF(B2&gt;0,B17/B2,0)</f>
         <v/>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajoute le brunch du lendemain (mariages) et le repas de cohésion (entreprises)
Page événements privés, formulaire de devis, plaquette et modèles d'e-mails.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZLSKwfEZhmFaHDXKS8XKA
</commit_message>
<xml_diff>
--- a/prospection/Yummy_Prospection_Evenements.xlsx
+++ b/prospection/Yummy_Prospection_Evenements.xlsx
@@ -2780,7 +2780,7 @@
         <is>
           <t>Bonjour,
 Nous sommes Yummy Street Food, le food truck vert de Virton : une street-food végétale préparée avec les légumes que nous cultivons nous-mêmes.
-Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail, nous proposons une formule de 3 ou 5 starters végétaux, puis un plat street food (burger ou pita) et un dessert si vous le souhaitez. Nous pouvons aussi assurer un service en fin de soirée.
+Nous aimerions faire partie des prestataires que vous recommandez à vos clients. Pour un vin d'honneur ou un cocktail, nous proposons une formule de 3 ou 5 starters végétaux, puis un plat street food (burger ou pita) et un dessert si vous le souhaitez. Nous pouvons aussi assurer un service en fin de soirée, et même le brunch du lendemain.
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf
 Le plus simple est encore de goûter : nous pouvons passer vous déposer un plateau de starters, à vous de nous dire quand.
 Toutes nos formules : https://yummy-streetfood.be/evenements-prives?src=lieux
@@ -2806,7 +2806,7 @@
         <is>
           <t>Bonjour {prénom},
 J'ai découvert votre travail et votre approche des mariages, et je pense que nous pourrions faire de beaux mariages ensemble.
-Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : starters en ouverture, puis burgers et pitas, avec les légumes de notre potager en Gaume. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
+Yummy Street Food, c'est une remorque vert émeraude et une cuisine végétale, locale et colorée : starters en ouverture, puis burgers et pitas, avec les légumes de notre potager en Gaume, et même le brunch du lendemain. Le résultat est aussi joli que bon, ce qui compte pour vos couples.
 Seriez-vous partant(e) pour un café et une dégustation ? Et bien sûr, nous recommandons volontiers vos services à nos clients en retour.
 Notre offre mariage : https://yummy-streetfood.be/evenements-prives?src=planners
 Au plaisir,
@@ -2830,10 +2830,10 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Bonjour {prénom},
-Vous préparez peut-être déjà la fête du personnel, un family day ou un séminaire pour 2027 ?
+Vous préparez peut-être déjà la fête du personnel, un repas de cohésion, un family day ou un séminaire pour 2027 ?
 Yummy Street Food est un food truck basé à Virton. Nous cuisinons une street-food végétale et gourmande avec les légumes de notre propre potager. Concrètement, la remorque s'installe sur votre site et sert vos équipes rapidement, sans qu'il y ait rien à organiser de votre côté.
 Nous proposons par exemple :
-- un lunch d'équipe ou une pause midi sur le parking ;
+- un repas de cohésion ou un lunch d'équipe, servi sur votre site ;
 - un apéro avec une formule de 3 ou 5 starters végétaux ;
 - un repas complet pour une fête du personnel ou un family day.
 Notre plaquette : https://yummy-streetfood.be/plaquette-evenements-yummy.pdf

</xml_diff>